<commit_message>
add Database Planning exercise
</commit_message>
<xml_diff>
--- a/W3/NormalizationChallenge.xlsx
+++ b/W3/NormalizationChallenge.xlsx
@@ -8,12 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RichardHawkins\Revature\2370-2371-DF-AI\trainer-code\W3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D03B257B-A2DD-4961-87D3-791B65384B30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5DD7071-A3F6-4528-8447-DDF623BB35AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="3120" windowWidth="21600" windowHeight="11295" xr2:uid="{411B24FF-7841-4CC7-ACDF-09F9293A7803}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{411B24FF-7841-4CC7-ACDF-09F9293A7803}"/>
   </bookViews>
   <sheets>
     <sheet name="NormalizationChallenge" sheetId="1" r:id="rId1"/>
+    <sheet name=".5NF" sheetId="6" r:id="rId2"/>
+    <sheet name="1NF" sheetId="2" r:id="rId3"/>
+    <sheet name="2NF" sheetId="3" r:id="rId4"/>
+    <sheet name="2NF (2)" sheetId="4" r:id="rId5"/>
+    <sheet name="3NF" sheetId="5" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="81">
   <si>
     <t>StudentID</t>
   </si>
@@ -138,6 +143,147 @@
   </si>
   <si>
     <t>B, B</t>
+  </si>
+  <si>
+    <t>CS101 (Intro to Java)</t>
+  </si>
+  <si>
+    <t>Prof. Aris (Rm 402)</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>BIO50 (Genetics)</t>
+  </si>
+  <si>
+    <t>Prof. Pierce (Rm 330)</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>MA205 (Calculus II)</t>
+  </si>
+  <si>
+    <t>Prof. Gauss (Rm 112)</t>
+  </si>
+  <si>
+    <t>B+</t>
+  </si>
+  <si>
+    <t>PY101 (Intro to Python)</t>
+  </si>
+  <si>
+    <t>Prof. Hopper (Rm 201)</t>
+  </si>
+  <si>
+    <t>PH200 (Mechanics)</t>
+  </si>
+  <si>
+    <t>Prof. Curie (Rm 505)</t>
+  </si>
+  <si>
+    <t>CPK</t>
+  </si>
+  <si>
+    <t>PK</t>
+  </si>
+  <si>
+    <t>Courses ID</t>
+  </si>
+  <si>
+    <t>Courses Titles</t>
+  </si>
+  <si>
+    <t>Courses IDs</t>
+  </si>
+  <si>
+    <t>Instructors</t>
+  </si>
+  <si>
+    <t>Offices</t>
+  </si>
+  <si>
+    <t>CS101</t>
+  </si>
+  <si>
+    <t>PL101</t>
+  </si>
+  <si>
+    <t>BIO50</t>
+  </si>
+  <si>
+    <t>MA205</t>
+  </si>
+  <si>
+    <t>PY101</t>
+  </si>
+  <si>
+    <t>PH200</t>
+  </si>
+  <si>
+    <t>Intro to Java</t>
+  </si>
+  <si>
+    <t>Ethics 101</t>
+  </si>
+  <si>
+    <t>Genetics</t>
+  </si>
+  <si>
+    <t>Calculus II</t>
+  </si>
+  <si>
+    <t>Intro to Python</t>
+  </si>
+  <si>
+    <t>Mechanics</t>
+  </si>
+  <si>
+    <t>Prof. Curie</t>
+  </si>
+  <si>
+    <t>Prof. Hopper</t>
+  </si>
+  <si>
+    <t>Prof. Gauss</t>
+  </si>
+  <si>
+    <t>Prof. Pierce</t>
+  </si>
+  <si>
+    <t>Prof. Specter</t>
+  </si>
+  <si>
+    <t>Prof. Aris</t>
+  </si>
+  <si>
+    <t>Rm 402</t>
+  </si>
+  <si>
+    <t>Rm 905</t>
+  </si>
+  <si>
+    <t>Rm 330</t>
+  </si>
+  <si>
+    <t>Rm 112</t>
+  </si>
+  <si>
+    <t>Rm 201</t>
+  </si>
+  <si>
+    <t>Rm 505</t>
+  </si>
+  <si>
+    <t>PARTIAL DEPENDENCY</t>
+  </si>
+  <si>
+    <t>TRANSITIVE DEPENDENCY</t>
   </si>
 </sst>
 </file>
@@ -549,154 +695,1746 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66EDA7C0-8AB6-474E-973F-5C73EBE5BC2B}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="49.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="48.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="1">
+        <v>1001</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="1">
+        <v>1002</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
+        <v>1003</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
+        <v>1004</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
+        <v>1005</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
+        <v>1006</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A48AC049-CF7E-4B97-A867-BC5AAE9CC769}">
+  <dimension ref="A1:F14"/>
+  <sheetFormatPr defaultColWidth="51" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="8.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="114.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="1">
+    <row r="3" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="1">
         <v>1001</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="1">
+      <c r="D3" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="1">
         <v>1002</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F4" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="114.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="1">
+    <row r="5" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
         <v>1003</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B5" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="129" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="1">
+      <c r="D5" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
         <v>1004</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B6" s="3" t="s">
         <v>21</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="171.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="1">
-        <v>1005</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>25</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>7</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="114.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
+        <v>1005</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
         <v>1006</v>
       </c>
+      <c r="B8" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="1">
+        <v>1001</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="1">
+        <v>1003</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="1">
+        <v>1004</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="1">
+        <v>1005</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="1">
+        <v>1005</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="1">
+        <v>1006</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{869B67AE-419C-481B-8E45-56B6F3ACD24E}">
+  <dimension ref="A1:H14"/>
+  <sheetFormatPr defaultColWidth="51" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.7109375" customWidth="1"/>
+    <col min="5" max="5" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="25" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="1">
+        <v>1001</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="1">
+        <v>1001</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="1">
+        <v>1002</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="1">
+        <v>1002</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
+        <v>1003</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" s="1">
+        <v>1003</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
+        <v>1004</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" s="1">
+        <v>1004</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
+        <v>1005</v>
+      </c>
       <c r="B7" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" s="1">
+        <v>1005</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
+        <v>1006</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>29</v>
       </c>
+      <c r="C8" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E8" s="1">
+        <v>1006</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E9" s="1">
+        <v>1001</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E10" s="1">
+        <v>1003</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E11" s="1">
+        <v>1004</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E12" s="1">
+        <v>1005</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E13" s="1">
+        <v>1005</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E14" s="1">
+        <v>1006</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5578762B-B726-4A80-A7F0-97D90C3164ED}">
+  <dimension ref="A1:J17"/>
+  <sheetFormatPr defaultColWidth="51" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.7109375" customWidth="1"/>
+    <col min="5" max="5" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="25" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.7109375" customWidth="1"/>
+    <col min="9" max="9" width="25" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="24.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F1" t="s">
+        <v>48</v>
+      </c>
+      <c r="I1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="1">
+        <v>1001</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="1">
+        <v>1001</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="1">
+        <v>1002</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="1">
+        <v>1002</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
+        <v>1003</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" s="1">
+        <v>1003</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
+        <v>1004</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" s="1">
+        <v>1004</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
+        <v>1005</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>25</v>
+      </c>
       <c r="C7" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" s="1">
+        <v>1005</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
+        <v>1006</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D7" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>33</v>
+      <c r="E8" s="1">
+        <v>1006</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E9" s="1">
+        <v>1001</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E10" s="1">
+        <v>1003</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E11" s="1">
+        <v>1004</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E12" s="1">
+        <v>1005</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E13" s="1">
+        <v>1005</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E14" s="1">
+        <v>1006</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>79</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8B92C4F-B3C6-4541-88FF-7E46EF8F6D8F}">
+  <dimension ref="A1:M14"/>
+  <sheetFormatPr defaultColWidth="51" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.7109375" customWidth="1"/>
+    <col min="5" max="5" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.7109375" customWidth="1"/>
+    <col min="10" max="10" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F1" t="s">
+        <v>48</v>
+      </c>
+      <c r="J1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="1">
+        <v>1001</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="1">
+        <v>1001</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="M3" s="3" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="1">
+        <v>1002</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="1">
+        <v>1002</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="M4" s="3" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
+        <v>1003</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" s="1">
+        <v>1003</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="M5" s="3" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
+        <v>1004</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" s="1">
+        <v>1004</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="L6" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="M6" s="3" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
+        <v>1005</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" s="1">
+        <v>1005</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="K7" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="L7" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="M7" s="3" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
+        <v>1006</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E8" s="1">
+        <v>1006</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="L8" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="M8" s="3" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E9" s="1">
+        <v>1001</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E10" s="1">
+        <v>1003</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E11" s="1">
+        <v>1004</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E12" s="1">
+        <v>1005</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E13" s="1">
+        <v>1005</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E14" s="1">
+        <v>1006</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD1A2FF8-D0E1-413F-9EE0-10178ED45C0D}">
+  <dimension ref="A1:N17"/>
+  <sheetFormatPr defaultColWidth="51" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.7109375" customWidth="1"/>
+    <col min="5" max="5" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.7109375" customWidth="1"/>
+    <col min="9" max="9" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.7109375" customWidth="1"/>
+    <col min="13" max="13" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F1" t="s">
+        <v>48</v>
+      </c>
+      <c r="I1" t="s">
+        <v>49</v>
+      </c>
+      <c r="M1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="1">
+        <v>1001</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="1">
+        <v>1001</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="M3" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="N3" s="3" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="1">
+        <v>1002</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="1">
+        <v>1002</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="M4" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="N4" s="3" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
+        <v>1003</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" s="1">
+        <v>1003</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="M5" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="N5" s="3" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
+        <v>1004</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" s="1">
+        <v>1004</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="M6" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="N6" s="3" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
+        <v>1005</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" s="1">
+        <v>1005</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="K7" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="M7" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="N7" s="3" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
+        <v>1006</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E8" s="1">
+        <v>1006</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="M8" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="N8" s="3" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E9" s="1">
+        <v>1001</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E10" s="1">
+        <v>1003</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E11" s="1">
+        <v>1004</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E12" s="1">
+        <v>1005</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E13" s="1">
+        <v>1005</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E14" s="1">
+        <v>1006</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>